<commit_message>
updated GSC export data
</commit_message>
<xml_diff>
--- a/gsc-export/Breadcrumbs.xlsx
+++ b/gsc-export/Breadcrumbs.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="95">
   <si>
     <t>Date</t>
   </si>
@@ -25,39 +25,6 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>2026-06-12</t>
-  </si>
-  <si>
-    <t>2026-06-13</t>
-  </si>
-  <si>
-    <t>2026-06-14</t>
-  </si>
-  <si>
-    <t>2026-06-15</t>
-  </si>
-  <si>
-    <t>2026-06-16</t>
-  </si>
-  <si>
-    <t>2026-06-17</t>
-  </si>
-  <si>
-    <t>2026-06-18</t>
-  </si>
-  <si>
-    <t>2026-06-19</t>
-  </si>
-  <si>
-    <t>2026-06-20</t>
-  </si>
-  <si>
-    <t>2026-06-21</t>
-  </si>
-  <si>
-    <t>2026-06-22</t>
-  </si>
-  <si>
     <t>2026-06-23</t>
   </si>
   <si>
@@ -293,6 +260,36 @@
   </si>
   <si>
     <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>2026-09-10</t>
+  </si>
+  <si>
+    <t>2026-09-11</t>
+  </si>
+  <si>
+    <t>2026-09-12</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>2026-09-16</t>
+  </si>
+  <si>
+    <t>2026-09-17</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>2026-09-19</t>
   </si>
   <si>
     <t>Issue</t>
@@ -351,7 +348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -373,7 +370,7 @@
         <v>0.0</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>52.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="3">
@@ -384,7 +381,7 @@
         <v>0.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>52.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="4">
@@ -395,7 +392,7 @@
         <v>0.0</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>52.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="5">
@@ -406,7 +403,7 @@
         <v>0.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>52.0</v>
+        <v>63.0</v>
       </c>
     </row>
     <row r="6">
@@ -417,7 +414,7 @@
         <v>0.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>54.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="7">
@@ -428,7 +425,7 @@
         <v>0.0</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>54.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="8">
@@ -439,7 +436,7 @@
         <v>0.0</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>56.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="9">
@@ -450,7 +447,7 @@
         <v>0.0</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>56.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="10">
@@ -461,7 +458,7 @@
         <v>0.0</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>56.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="11">
@@ -472,7 +469,7 @@
         <v>0.0</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>60.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="12">
@@ -483,7 +480,7 @@
         <v>0.0</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>62.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="13">
@@ -505,7 +502,7 @@
         <v>0.0</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>64.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="15">
@@ -516,7 +513,7 @@
         <v>0.0</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>64.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="16">
@@ -527,7 +524,7 @@
         <v>0.0</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>63.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="17">
@@ -538,7 +535,7 @@
         <v>0.0</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>65.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="18">
@@ -549,7 +546,7 @@
         <v>0.0</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>65.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="19">
@@ -560,7 +557,7 @@
         <v>0.0</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="20">
@@ -571,7 +568,7 @@
         <v>0.0</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>65.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="21">
@@ -582,7 +579,7 @@
         <v>0.0</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="22">
@@ -593,7 +590,7 @@
         <v>0.0</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="23">
@@ -604,7 +601,7 @@
         <v>0.0</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="24">
@@ -615,7 +612,7 @@
         <v>0.0</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>64.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="25">
@@ -626,7 +623,7 @@
         <v>0.0</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>65.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="26">
@@ -637,7 +634,7 @@
         <v>0.0</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>66.0</v>
+        <v>69.0</v>
       </c>
     </row>
     <row r="27">
@@ -648,7 +645,7 @@
         <v>0.0</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>66.0</v>
+        <v>70.0</v>
       </c>
     </row>
     <row r="28">
@@ -659,7 +656,7 @@
         <v>0.0</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>66.0</v>
+        <v>72.0</v>
       </c>
     </row>
     <row r="29">
@@ -670,7 +667,7 @@
         <v>0.0</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>67.0</v>
+        <v>72.0</v>
       </c>
     </row>
     <row r="30">
@@ -681,7 +678,7 @@
         <v>0.0</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>67.0</v>
+        <v>71.0</v>
       </c>
     </row>
     <row r="31">
@@ -692,7 +689,7 @@
         <v>0.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>68.0</v>
+        <v>71.0</v>
       </c>
     </row>
     <row r="32">
@@ -703,7 +700,7 @@
         <v>0.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>67.0</v>
+        <v>71.0</v>
       </c>
     </row>
     <row r="33">
@@ -714,7 +711,7 @@
         <v>0.0</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>67.0</v>
+        <v>71.0</v>
       </c>
     </row>
     <row r="34">
@@ -725,7 +722,7 @@
         <v>0.0</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>67.0</v>
+        <v>69.0</v>
       </c>
     </row>
     <row r="35">
@@ -736,7 +733,7 @@
         <v>0.0</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>68.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="36">
@@ -747,7 +744,7 @@
         <v>0.0</v>
       </c>
       <c r="C36" t="n" s="0">
-        <v>68.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="37">
@@ -758,7 +755,7 @@
         <v>0.0</v>
       </c>
       <c r="C37" t="n" s="0">
-        <v>69.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="38">
@@ -769,7 +766,7 @@
         <v>0.0</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>70.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="39">
@@ -780,7 +777,7 @@
         <v>0.0</v>
       </c>
       <c r="C39" t="n" s="0">
-        <v>72.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="40">
@@ -791,7 +788,7 @@
         <v>0.0</v>
       </c>
       <c r="C40" t="n" s="0">
-        <v>72.0</v>
+        <v>63.0</v>
       </c>
     </row>
     <row r="41">
@@ -802,7 +799,7 @@
         <v>0.0</v>
       </c>
       <c r="C41" t="n" s="0">
-        <v>71.0</v>
+        <v>61.0</v>
       </c>
     </row>
     <row r="42">
@@ -813,7 +810,7 @@
         <v>0.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>71.0</v>
+        <v>58.0</v>
       </c>
     </row>
     <row r="43">
@@ -824,7 +821,7 @@
         <v>0.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>71.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="44">
@@ -835,7 +832,7 @@
         <v>0.0</v>
       </c>
       <c r="C44" t="n" s="0">
-        <v>71.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="45">
@@ -846,7 +843,7 @@
         <v>0.0</v>
       </c>
       <c r="C45" t="n" s="0">
-        <v>69.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="46">
@@ -857,7 +854,7 @@
         <v>0.0</v>
       </c>
       <c r="C46" t="n" s="0">
-        <v>67.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="47">
@@ -868,7 +865,7 @@
         <v>0.0</v>
       </c>
       <c r="C47" t="n" s="0">
-        <v>67.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="48">
@@ -879,7 +876,7 @@
         <v>0.0</v>
       </c>
       <c r="C48" t="n" s="0">
-        <v>66.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="49">
@@ -890,7 +887,7 @@
         <v>0.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>66.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="50">
@@ -901,7 +898,7 @@
         <v>0.0</v>
       </c>
       <c r="C50" t="n" s="0">
-        <v>66.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="51">
@@ -912,7 +909,7 @@
         <v>0.0</v>
       </c>
       <c r="C51" t="n" s="0">
-        <v>63.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="52">
@@ -923,7 +920,7 @@
         <v>0.0</v>
       </c>
       <c r="C52" t="n" s="0">
-        <v>61.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="53">
@@ -934,7 +931,7 @@
         <v>0.0</v>
       </c>
       <c r="C53" t="n" s="0">
-        <v>58.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="54">
@@ -956,7 +953,7 @@
         <v>0.0</v>
       </c>
       <c r="C55" t="n" s="0">
-        <v>57.0</v>
+        <v>55.0</v>
       </c>
     </row>
     <row r="56">
@@ -967,7 +964,7 @@
         <v>0.0</v>
       </c>
       <c r="C56" t="n" s="0">
-        <v>57.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="57">
@@ -978,7 +975,7 @@
         <v>0.0</v>
       </c>
       <c r="C57" t="n" s="0">
-        <v>57.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="58">
@@ -989,7 +986,7 @@
         <v>0.0</v>
       </c>
       <c r="C58" t="n" s="0">
-        <v>57.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="59">
@@ -1000,7 +997,7 @@
         <v>0.0</v>
       </c>
       <c r="C59" t="n" s="0">
-        <v>57.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="60">
@@ -1011,7 +1008,7 @@
         <v>0.0</v>
       </c>
       <c r="C60" t="n" s="0">
-        <v>57.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="61">
@@ -1022,7 +1019,7 @@
         <v>0.0</v>
       </c>
       <c r="C61" t="n" s="0">
-        <v>57.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="62">
@@ -1033,7 +1030,7 @@
         <v>0.0</v>
       </c>
       <c r="C62" t="n" s="0">
-        <v>57.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="63">
@@ -1044,7 +1041,7 @@
         <v>0.0</v>
       </c>
       <c r="C63" t="n" s="0">
-        <v>57.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="64">
@@ -1055,7 +1052,7 @@
         <v>0.0</v>
       </c>
       <c r="C64" t="n" s="0">
-        <v>57.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="65">
@@ -1066,7 +1063,7 @@
         <v>0.0</v>
       </c>
       <c r="C65" t="n" s="0">
-        <v>57.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="66">
@@ -1077,7 +1074,7 @@
         <v>0.0</v>
       </c>
       <c r="C66" t="n" s="0">
-        <v>55.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="67">
@@ -1088,7 +1085,7 @@
         <v>0.0</v>
       </c>
       <c r="C67" t="n" s="0">
-        <v>54.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="68">
@@ -1099,7 +1096,7 @@
         <v>0.0</v>
       </c>
       <c r="C68" t="n" s="0">
-        <v>54.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="69">
@@ -1110,7 +1107,7 @@
         <v>0.0</v>
       </c>
       <c r="C69" t="n" s="0">
-        <v>54.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="70">
@@ -1121,7 +1118,7 @@
         <v>0.0</v>
       </c>
       <c r="C70" t="n" s="0">
-        <v>54.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="71">
@@ -1143,7 +1140,7 @@
         <v>0.0</v>
       </c>
       <c r="C72" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="73">
@@ -1154,7 +1151,7 @@
         <v>0.0</v>
       </c>
       <c r="C73" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="74">
@@ -1165,7 +1162,7 @@
         <v>0.0</v>
       </c>
       <c r="C74" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="75">
@@ -1176,7 +1173,7 @@
         <v>0.0</v>
       </c>
       <c r="C75" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="76">
@@ -1198,7 +1195,7 @@
         <v>0.0</v>
       </c>
       <c r="C77" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="78">
@@ -1209,7 +1206,7 @@
         <v>0.0</v>
       </c>
       <c r="C78" t="n" s="0">
-        <v>52.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="79">
@@ -1220,7 +1217,7 @@
         <v>0.0</v>
       </c>
       <c r="C79" t="n" s="0">
-        <v>52.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="80">
@@ -1231,7 +1228,7 @@
         <v>0.0</v>
       </c>
       <c r="C80" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="81">
@@ -1242,7 +1239,7 @@
         <v>0.0</v>
       </c>
       <c r="C81" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="82">
@@ -1253,7 +1250,7 @@
         <v>0.0</v>
       </c>
       <c r="C82" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="83">
@@ -1264,7 +1261,7 @@
         <v>0.0</v>
       </c>
       <c r="C83" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="84">
@@ -1275,7 +1272,7 @@
         <v>0.0</v>
       </c>
       <c r="C84" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="85">
@@ -1286,7 +1283,7 @@
         <v>0.0</v>
       </c>
       <c r="C85" t="n" s="0">
-        <v>53.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="86">
@@ -1308,7 +1305,7 @@
         <v>0.0</v>
       </c>
       <c r="C87" t="n" s="0">
-        <v>52.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="88">
@@ -1330,7 +1327,7 @@
         <v>0.0</v>
       </c>
       <c r="C89" t="n" s="0">
-        <v>54.0</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="90">
@@ -1341,18 +1338,7 @@
         <v>0.0</v>
       </c>
       <c r="C90" t="n" s="0">
-        <v>54.0</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="B91" t="n" s="0">
-        <v>0.0</v>
-      </c>
-      <c r="C91" t="n" s="0">
-        <v>54.0</v>
+        <v>53.0</v>
       </c>
     </row>
   </sheetData>
@@ -1367,13 +1353,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s" s="0">
         <v>93</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="C1" t="s" s="0">
         <v>94</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1388,13 +1374,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s" s="0">
         <v>93</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="C1" t="s" s="0">
         <v>94</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>